<commit_message>
Add logging configuration, tests, and update Arbiter mappings
- Introduced logging configuration in `logging_config.py` for better logging management.
- Added unit tests for `ArbiterOperations` in `test_arbiter_ops.py` and `test_arbiter_ops_mapping.py` to ensure functionality.
- Updated Arbiter mappings by replacing the old Excel file with a new version and removing temporary files.
- Created a new game import template for 2025-10.
- Implemented a runner script `run_arbiter.py` to facilitate execution of the `ArbiterOperations` process.
</commit_message>
<xml_diff>
--- a/arbiter_etl/data/fall2025/lookup/ArbiterMappings.xlsx
+++ b/arbiter_etl/data/fall2025/lookup/ArbiterMappings.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10119"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10810"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/roxberry/Workspaces/SJSL/gotsport-toolbox/arbiter_etl/data/spring2025/lookup/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/roxberry/Workspaces/SJSL/gotsport-toolbox/arbiter_etl/data/fall2025/lookup/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DFB786A7-FC14-0844-A178-DF728AB5548E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{61C3CFB7-3273-9E46-B13F-523508CC6116}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="760" windowWidth="34560" windowHeight="21580" activeTab="1" xr2:uid="{560EA3F1-29A7-EA41-B41C-8BD96A0307DA}"/>
+    <workbookView xWindow="0" yWindow="680" windowWidth="34560" windowHeight="20120" activeTab="2" xr2:uid="{560EA3F1-29A7-EA41-B41C-8BD96A0307DA}"/>
   </bookViews>
   <sheets>
     <sheet name="LevelsMap" sheetId="1" r:id="rId1"/>
@@ -43,7 +43,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="731" uniqueCount="716">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="751" uniqueCount="733">
   <si>
     <t>U8</t>
   </si>
@@ -2191,13 +2191,64 @@
   </si>
   <si>
     <t>WTYSA - Peter Volpa Park</t>
+  </si>
+  <si>
+    <t>Cherry Hill East HS</t>
+  </si>
+  <si>
+    <t>CHERRY HILL EAST HS</t>
+  </si>
+  <si>
+    <t>Delran FC-Peter Vermes Fields</t>
+  </si>
+  <si>
+    <t>DELRAN - VERMES</t>
+  </si>
+  <si>
+    <t>EPAA-Weimann Sports Complex</t>
+  </si>
+  <si>
+    <t>EPAA - Weimann Sports Complex</t>
+  </si>
+  <si>
+    <t>Haddon Twp - Van Sciver School</t>
+  </si>
+  <si>
+    <t>HADDON TWP - VAN SCIVER SCHOOL</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Northern Burlington - Mansfield Georgetown </t>
+  </si>
+  <si>
+    <t>PRSC - Riverton Park</t>
+  </si>
+  <si>
+    <t>PAL RIV - Riverton Park Fall Season</t>
+  </si>
+  <si>
+    <t>South Harrison - Stewart Park</t>
+  </si>
+  <si>
+    <t>SOUTH HARRISON - STEWART</t>
+  </si>
+  <si>
+    <t>Waterford Elementary School</t>
+  </si>
+  <si>
+    <t>WATERFORD - ELEMENTARY SCHOOL</t>
+  </si>
+  <si>
+    <t>WTYSA  - Peter Volpa Park</t>
+  </si>
+  <si>
+    <t>WTSC Levy Memorial Fields</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="5" x14ac:knownFonts="1">
+  <fonts count="6" x14ac:knownFonts="1">
     <font>
       <sz val="12"/>
       <color theme="1"/>
@@ -2235,6 +2286,12 @@
       <family val="2"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <sz val="12"/>
+      <color rgb="FF333333"/>
+      <name val="Arial"/>
+      <family val="2"/>
+    </font>
   </fonts>
   <fills count="2">
     <fill>
@@ -2256,7 +2313,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="6">
+  <cellXfs count="7">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
@@ -2265,6 +2322,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -6599,6 +6657,86 @@
         <v>244</v>
       </c>
     </row>
+    <row r="79" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A79" t="s">
+        <v>716</v>
+      </c>
+      <c r="B79" s="6" t="s">
+        <v>717</v>
+      </c>
+    </row>
+    <row r="80" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A80" t="s">
+        <v>718</v>
+      </c>
+      <c r="B80" s="6" t="s">
+        <v>719</v>
+      </c>
+    </row>
+    <row r="81" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A81" t="s">
+        <v>720</v>
+      </c>
+      <c r="B81" s="6" t="s">
+        <v>721</v>
+      </c>
+    </row>
+    <row r="82" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A82" t="s">
+        <v>722</v>
+      </c>
+      <c r="B82" s="6" t="s">
+        <v>723</v>
+      </c>
+    </row>
+    <row r="83" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A83" t="s">
+        <v>724</v>
+      </c>
+      <c r="B83" s="6" t="s">
+        <v>701</v>
+      </c>
+    </row>
+    <row r="84" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A84" t="s">
+        <v>725</v>
+      </c>
+      <c r="B84" s="6" t="s">
+        <v>726</v>
+      </c>
+    </row>
+    <row r="85" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A85" t="s">
+        <v>727</v>
+      </c>
+      <c r="B85" s="6" t="s">
+        <v>728</v>
+      </c>
+    </row>
+    <row r="86" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A86" t="s">
+        <v>729</v>
+      </c>
+      <c r="B86" s="6" t="s">
+        <v>730</v>
+      </c>
+    </row>
+    <row r="87" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A87" t="s">
+        <v>731</v>
+      </c>
+      <c r="B87" t="s">
+        <v>244</v>
+      </c>
+    </row>
+    <row r="88" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A88" t="s">
+        <v>732</v>
+      </c>
+      <c r="B88" t="s">
+        <v>242</v>
+      </c>
+    </row>
     <row r="119" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A119" s="5"/>
     </row>

</xml_diff>